<commit_message>
daily auto push: 2026-07-21 15:15 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D782"/>
+  <dimension ref="A1:D783"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14403,16 +14403,16 @@
     <row r="777">
       <c r="A777" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/07/20</t>
         </is>
       </c>
       <c r="B777" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C777" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D777" t="n">
         <v>101</v>
@@ -14421,12 +14421,12 @@
     <row r="778">
       <c r="A778" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B778" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C778" t="n">
@@ -14439,12 +14439,12 @@
     <row r="779">
       <c r="A779" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B779" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C779" t="n">
@@ -14457,12 +14457,12 @@
     <row r="780">
       <c r="A780" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B780" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C780" t="n">
@@ -14475,12 +14475,12 @@
     <row r="781">
       <c r="A781" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B781" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C781" t="n">
@@ -14493,18 +14493,36 @@
     <row r="782">
       <c r="A782" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C782" t="n">
+        <v>22</v>
+      </c>
+      <c r="D782" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B782" t="inlineStr">
+      <c r="B783" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C782" t="n">
-        <v>22</v>
-      </c>
-      <c r="D782" t="n">
+      <c r="C783" t="n">
+        <v>22</v>
+      </c>
+      <c r="D783" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-30 12:49 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D822"/>
+  <dimension ref="A1:D823"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15123,16 +15123,16 @@
     <row r="817">
       <c r="A817" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/29</t>
         </is>
       </c>
       <c r="B817" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C817" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D817" t="n">
         <v>101</v>
@@ -15141,12 +15141,12 @@
     <row r="818">
       <c r="A818" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B818" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C818" t="n">
@@ -15159,12 +15159,12 @@
     <row r="819">
       <c r="A819" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B819" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C819" t="n">
@@ -15177,12 +15177,12 @@
     <row r="820">
       <c r="A820" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B820" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C820" t="n">
@@ -15195,12 +15195,12 @@
     <row r="821">
       <c r="A821" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B821" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C821" t="n">
@@ -15213,18 +15213,36 @@
     <row r="822">
       <c r="A822" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C822" t="n">
+        <v>22</v>
+      </c>
+      <c r="D822" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B822" t="inlineStr">
+      <c r="B823" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C822" t="n">
-        <v>22</v>
-      </c>
-      <c r="D822" t="n">
+      <c r="C823" t="n">
+        <v>22</v>
+      </c>
+      <c r="D823" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-02 12:04 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D825"/>
+  <dimension ref="A1:D826"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15177,7 +15177,7 @@
     <row r="820">
       <c r="A820" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/01</t>
         </is>
       </c>
       <c r="B820" t="inlineStr">
@@ -15186,7 +15186,7 @@
         </is>
       </c>
       <c r="C820" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D820" t="n">
         <v>101</v>
@@ -15195,12 +15195,12 @@
     <row r="821">
       <c r="A821" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B821" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C821" t="n">
@@ -15213,12 +15213,12 @@
     <row r="822">
       <c r="A822" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B822" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C822" t="n">
@@ -15231,12 +15231,12 @@
     <row r="823">
       <c r="A823" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C823" t="n">
@@ -15249,12 +15249,12 @@
     <row r="824">
       <c r="A824" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C824" t="n">
@@ -15267,18 +15267,36 @@
     <row r="825">
       <c r="A825" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C825" t="n">
+        <v>22</v>
+      </c>
+      <c r="D825" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B825" t="inlineStr">
+      <c r="B826" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C825" t="n">
-        <v>22</v>
-      </c>
-      <c r="D825" t="n">
+      <c r="C826" t="n">
+        <v>22</v>
+      </c>
+      <c r="D826" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-03 12:04 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D826"/>
+  <dimension ref="A1:D827"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15195,16 +15195,16 @@
     <row r="821">
       <c r="A821" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/02</t>
         </is>
       </c>
       <c r="B821" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C821" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D821" t="n">
         <v>101</v>
@@ -15213,12 +15213,12 @@
     <row r="822">
       <c r="A822" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B822" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C822" t="n">
@@ -15231,12 +15231,12 @@
     <row r="823">
       <c r="A823" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C823" t="n">
@@ -15249,12 +15249,12 @@
     <row r="824">
       <c r="A824" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C824" t="n">
@@ -15267,12 +15267,12 @@
     <row r="825">
       <c r="A825" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B825" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C825" t="n">
@@ -15285,18 +15285,36 @@
     <row r="826">
       <c r="A826" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C826" t="n">
+        <v>22</v>
+      </c>
+      <c r="D826" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B826" t="inlineStr">
+      <c r="B827" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C826" t="n">
-        <v>22</v>
-      </c>
-      <c r="D826" t="n">
+      <c r="C827" t="n">
+        <v>22</v>
+      </c>
+      <c r="D827" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-06 12:50 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D829"/>
+  <dimension ref="A1:D830"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15249,16 +15249,16 @@
     <row r="824">
       <c r="A824" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/05</t>
         </is>
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C824" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D824" t="n">
         <v>101</v>
@@ -15267,12 +15267,12 @@
     <row r="825">
       <c r="A825" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B825" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C825" t="n">
@@ -15285,12 +15285,12 @@
     <row r="826">
       <c r="A826" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B826" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C826" t="n">
@@ -15303,12 +15303,12 @@
     <row r="827">
       <c r="A827" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B827" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C827" t="n">
@@ -15321,12 +15321,12 @@
     <row r="828">
       <c r="A828" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B828" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C828" t="n">
@@ -15339,18 +15339,36 @@
     <row r="829">
       <c r="A829" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C829" t="n">
+        <v>22</v>
+      </c>
+      <c r="D829" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B829" t="inlineStr">
+      <c r="B830" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C829" t="n">
-        <v>22</v>
-      </c>
-      <c r="D829" t="n">
+      <c r="C830" t="n">
+        <v>22</v>
+      </c>
+      <c r="D830" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-09 12:18 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D836"/>
+  <dimension ref="A1:D837"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15375,16 +15375,16 @@
     <row r="831">
       <c r="A831" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/09</t>
         </is>
       </c>
       <c r="B831" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C831" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D831" t="n">
         <v>101</v>
@@ -15393,12 +15393,12 @@
     <row r="832">
       <c r="A832" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B832" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C832" t="n">
@@ -15411,12 +15411,12 @@
     <row r="833">
       <c r="A833" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C833" t="n">
@@ -15429,12 +15429,12 @@
     <row r="834">
       <c r="A834" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B834" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C834" t="n">
@@ -15447,12 +15447,12 @@
     <row r="835">
       <c r="A835" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B835" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C835" t="n">
@@ -15465,18 +15465,36 @@
     <row r="836">
       <c r="A836" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C836" t="n">
+        <v>22</v>
+      </c>
+      <c r="D836" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B836" t="inlineStr">
+      <c r="B837" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C836" t="n">
-        <v>22</v>
-      </c>
-      <c r="D836" t="n">
+      <c r="C837" t="n">
+        <v>22</v>
+      </c>
+      <c r="D837" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-10 12:12 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D837"/>
+  <dimension ref="A1:D838"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15393,16 +15393,16 @@
     <row r="832">
       <c r="A832" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/09</t>
         </is>
       </c>
       <c r="B832" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C832" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D832" t="n">
         <v>101</v>
@@ -15411,12 +15411,12 @@
     <row r="833">
       <c r="A833" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C833" t="n">
@@ -15429,12 +15429,12 @@
     <row r="834">
       <c r="A834" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B834" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C834" t="n">
@@ -15447,12 +15447,12 @@
     <row r="835">
       <c r="A835" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B835" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C835" t="n">
@@ -15465,12 +15465,12 @@
     <row r="836">
       <c r="A836" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B836" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C836" t="n">
@@ -15483,18 +15483,36 @@
     <row r="837">
       <c r="A837" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C837" t="n">
+        <v>22</v>
+      </c>
+      <c r="D837" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B837" t="inlineStr">
+      <c r="B838" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C837" t="n">
-        <v>22</v>
-      </c>
-      <c r="D837" t="n">
+      <c r="C838" t="n">
+        <v>22</v>
+      </c>
+      <c r="D838" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-12 12:49 UTC
</commit_message>
<xml_diff>
--- a/excel/spotify.xlsx
+++ b/excel/spotify.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D843"/>
+  <dimension ref="A1:D844"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15501,16 +15501,16 @@
     <row r="838">
       <c r="A838" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/12</t>
         </is>
       </c>
       <c r="B838" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C838" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="D838" t="n">
         <v>101</v>
@@ -15519,12 +15519,12 @@
     <row r="839">
       <c r="A839" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B839" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C839" t="n">
@@ -15537,12 +15537,12 @@
     <row r="840">
       <c r="A840" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B840" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C840" t="n">
@@ -15555,12 +15555,12 @@
     <row r="841">
       <c r="A841" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B841" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C841" t="n">
@@ -15573,12 +15573,12 @@
     <row r="842">
       <c r="A842" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B842" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C842" t="n">
@@ -15591,18 +15591,36 @@
     <row r="843">
       <c r="A843" t="inlineStr">
         <is>
+          <t>2027/01/02</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C843" t="n">
+        <v>22</v>
+      </c>
+      <c r="D843" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
           <t>2027/01/03</t>
         </is>
       </c>
-      <c r="B843" t="inlineStr">
+      <c r="B844" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="C843" t="n">
-        <v>22</v>
-      </c>
-      <c r="D843" t="n">
+      <c r="C844" t="n">
+        <v>22</v>
+      </c>
+      <c r="D844" t="n">
         <v>101</v>
       </c>
     </row>

</xml_diff>